<commit_message>
Remove embedded personal paths from Excel metadata
Remove the saved personal storage path from both representative workbooks. Preserve all worksheet data, formatting, and author attribution.
</commit_message>
<xml_diff>
--- a/representative_data/MLTD collapsed.xlsx
+++ b/representative_data/MLTD collapsed.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tumde-my.sharepoint.com/personal/shanmugaraj_senthilnathan_tum_de/Documents/shan_old work/14. Monitoring control framework/5. MS journal submission/data availability/C3DP-MLTD-reproducability-data/representative_data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="17" documentId="11_AD4DB114E441178AC67DF444BED0D518683EDF2D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D16E3B4-9DB2-44EB-A6E5-CEE7F2BA6AAB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>